<commit_message>
Enhance compare-test and main.js to integrate findSameProjectPeers functionality. Update compare-test to validate ghost peer detection for deleted shifts and adjust main.js to utilize peerSchedule option in fillEventCard for improved event rendering. Update example shift file for testing purposes.
</commit_message>
<xml_diff>
--- a/example/shiftTotalTable0519_viki.xlsx
+++ b/example/shiftTotalTable0519_viki.xlsx
@@ -2274,8 +2274,8 @@
       <c r="AG1" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="AH1" s="5"/>
-      <c r="AI1" s="1"/>
+      <c r="AH1" s="4"/>
+      <c r="AI1" s="5"/>
       <c r="AJ1" s="1"/>
       <c r="AK1" s="17" t="s">
         <v>7</v>
@@ -58752,14 +58752,14 @@
     <mergeCell ref="U2:W2"/>
     <mergeCell ref="AC1:AE1"/>
     <mergeCell ref="AC2:AE2"/>
+    <mergeCell ref="D1:F1"/>
     <mergeCell ref="P1:R1"/>
+    <mergeCell ref="Z1:AA1"/>
     <mergeCell ref="C2:F2"/>
     <mergeCell ref="P2:R2"/>
     <mergeCell ref="Y2:AA2"/>
     <mergeCell ref="AF2:AG2"/>
-    <mergeCell ref="D1:F1"/>
-    <mergeCell ref="Z1:AA1"/>
-    <mergeCell ref="AG1:AH1"/>
+    <mergeCell ref="AG1:AI1"/>
     <mergeCell ref="H1:N1"/>
     <mergeCell ref="H2:N2"/>
     <mergeCell ref="C5:C7"/>

</xml_diff>